<commit_message>
jointure standardised species name à list_sp
</commit_message>
<xml_diff>
--- a/output/list_sp_clean.xlsx
+++ b/output/list_sp_clean.xlsx
@@ -351,7 +351,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B167"/>
+  <dimension ref="A1:B169"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -530,7 +530,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Bellis perennis</t>
+          <t>Bellis pèrennis</t>
         </is>
       </c>
     </row>
@@ -698,7 +698,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Carex hirsuta</t>
+          <t>Carex hirta</t>
         </is>
       </c>
     </row>
@@ -760,1574 +760,1598 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Carvul</t>
+          <t>Carlep</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Carex vulpina</t>
+          <t>Carex leporina</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Cenjac</t>
+          <t>Carvul</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Centaurea jacea</t>
+          <t>Carex vulpina</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Cerglo</t>
+          <t>Cenjac</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Cerastium glomeratum</t>
+          <t>Centaurea jacea</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Cerfon</t>
+          <t>Cerglo</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Cerastium fontanum</t>
+          <t>Cerastium glomeratum</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Cincri</t>
+          <t>Cerfon</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Cinosorus cristatus</t>
+          <t>Cerastium fontanum</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Cirsp</t>
+          <t>Cincri</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Cirsium sp.</t>
+          <t>Cinosorus cristatus</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Cirarv</t>
+          <t>Cirsp</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Cirsium arvense</t>
+          <t>Cirsium sp.</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Conarv</t>
+          <t>Cirarv</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Conyza arvensis</t>
+          <t>Cirsium arvense</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Convarv</t>
+          <t>Conarv</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Convolvulus arvensis</t>
+          <t>Conyza arvensis</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Cralae</t>
+          <t>Convarv</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Crataegus laevigata</t>
+          <t>Convolvulus arvensis</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Craoxy</t>
+          <t>Cralae</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Crataegus oxyacantha</t>
+          <t>Crataegus laevigata</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Crevir</t>
+          <t>Craoxy</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Crepis virens</t>
+          <t>Crataegus oxyacantha</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Crecap</t>
+          <t>Crevir</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Crepis capilaris</t>
+          <t>Crepis virens</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Cyncri</t>
+          <t>Crecap</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Cynosurus cristatus</t>
+          <t>Crepis capilaris</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Dacglo</t>
+          <t>Cyncri</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Dactylis glomerata</t>
+          <t>Cynosurus cristatus</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Dacinc</t>
+          <t>Dacglo</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Dactylorhiza incarnata</t>
+          <t>Dactylis glomerata</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Dacmac</t>
+          <t>Dacinc</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Dactylorhiza maculata</t>
+          <t>Dactylorhiza incarnata</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Daucar</t>
+          <t>Dacmac</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Daucus carota</t>
+          <t>Dactylorhiza maculata</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Decfle</t>
+          <t>Daucar</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Dechampsia flexuosa</t>
+          <t>Daucus carota</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Elepal</t>
+          <t>Decfle</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Eleocharis palustris</t>
+          <t>Dechampsia flexuosa</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Epihir</t>
+          <t>Elepal</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Epilobium hirsutum</t>
+          <t>Eleocharis palustris</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Episp</t>
+          <t>Epihir</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Epilobium sp.</t>
+          <t>Epilobium hirsutum</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Equarv</t>
+          <t>Episp</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Equisetum arvense</t>
+          <t>Epilobium sp.</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Feshec</t>
+          <t>Equarv</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Festuca heterophylla</t>
+          <t>Equisetum arvense</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Fesovi</t>
+          <t>Feshec</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Festuca ovina</t>
+          <t>Festuca heterophylla</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Fespra</t>
+          <t>Fesovi</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Festuca pratensis</t>
+          <t>Festuca ovina</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Fesrub</t>
+          <t>Fespra</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Festuca rubra</t>
+          <t>Festuca pratensis</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Fessp</t>
+          <t>Fesrub</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Festuca sp.</t>
+          <t>Festuca rubra</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Filulm</t>
+          <t>Fessp</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Filipendula ulmaria</t>
+          <t>Festuca sp.</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Galapa</t>
+          <t>Filulm</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>Gallium aparine</t>
+          <t>Filipendula ulmaria</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Galmol</t>
+          <t>Galapa</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Gallium mollugo</t>
+          <t>Gallium aparine</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>Galsp</t>
+          <t>Galmol</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>Galium sp.</t>
+          <t>Gallium mollugo</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>Galver</t>
+          <t>Galsp</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>Galium verum</t>
+          <t>Galium sp.</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>Gaufra</t>
+          <t>Galver</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>Gaudinia fragilis</t>
+          <t>Galium verum</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>Gercol</t>
+          <t>Gaufra</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>Geranium columbinum</t>
+          <t>Gaudinia fragilis</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>Gerdis</t>
+          <t>Gercol</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>Geranium dissectum</t>
+          <t>Geranium columbinum</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>Gerrob</t>
+          <t>Gerdis</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>Geranium robertianum</t>
+          <t>Geranium dissectum</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>Gersp</t>
+          <t>Gerrob</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>Geranium sp.</t>
+          <t>Geranium robertianum</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>Glehed</t>
+          <t>Gersp</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>Glecoma hederacea</t>
+          <t>Geranium sp.</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>Grasp</t>
+          <t>Glehed</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>Poacee inconnue</t>
+          <t>Glecoma hederacea</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>Hersib</t>
+          <t>Grasp</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>Heracleum sibiricum</t>
+          <t>Poacee inconnue</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>Hiesp</t>
+          <t>Hersib</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>Hiaracium sp.</t>
+          <t>Heracleum sibiricum</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>Hollan</t>
+          <t>Hiesp</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>Holcus lannatus</t>
+          <t>Hiaracium sp.</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>Hypper</t>
+          <t>Hollan</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>Hypericum perforatum</t>
+          <t>Holcus lannatus</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>Hyprad</t>
+          <t>Hypper</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>Hypochaeris radicata</t>
+          <t>Hypericum perforatum</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>inconnu</t>
+          <t>Hyprad</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>inconnu</t>
+          <t>Hypochaeris radicata</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>Juncus</t>
+          <t>inconnu</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>Juncus sp.</t>
+          <t>inconnu</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>Lamsp</t>
+          <t>Juncus</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>Lamiaceae sp.</t>
+          <t>Juncus sp.</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>Latarv</t>
+          <t>Lamsp</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>Lathyrus arvensis</t>
+          <t>Lamiaceae sp.</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>Lathyrus ochrus</t>
+          <t>Latarv</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>Lathyrus ochrus</t>
+          <t>Lathyrus arvensis</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>Latpra</t>
+          <t>Lathyrus ochrus</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>Lathyrus pratensis</t>
+          <t>Lathyrus ochrus</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>Latsat</t>
+          <t>Latpra</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>Lathyrus sativa</t>
+          <t>Lathyrus pratensis</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>Latsp</t>
+          <t>Latsat</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>Lathyrus sp</t>
+          <t>Lathyrus sativa</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>Leoaut</t>
+          <t>Latsp</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>Leontodon autumnalis</t>
+          <t>Lathyrus sp</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>Lepfil</t>
+          <t>Leoaut</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>Leontodon autumnalis</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>Leuvul</t>
-        </is>
-      </c>
-      <c r="B90" t="inlineStr">
-        <is>
-          <t>Leucanthemum vulgare</t>
+          <t>Lepfil</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>lincat</t>
+          <t>Leuvul</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>Linum catarthicum</t>
+          <t>Leucanthemum vulgare</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>LolIt</t>
+          <t>lincat</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>Lolium italicum</t>
+          <t>Linum catarthicum</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>Lolmul</t>
+          <t>LolIt</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>Lolium multiflorum (=Lolium italicum)</t>
+          <t>Lolium italicum</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>Lolper</t>
+          <t>Lolmul</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>Lolium perenne</t>
+          <t>Lolium multiflorum (=Lolium italicum)</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>Lolaru (=Fesaru)</t>
+          <t>Lolper</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>Lolium arundinaceum (=Festuca arundinacea)</t>
+          <t>Lolium pèrenne</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>Lotcor</t>
+          <t>Lolaru (=Fesaru)</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>Lotus corniculatus</t>
+          <t>Lolium arundinaceum (=Festuca arundinacea)</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>Lotped</t>
+          <t>Lotcor</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>Lotus pedunculatus</t>
+          <t>Lotus corniculatus</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>Lotuli</t>
+          <t>Lotped</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>Lotus uliginosus</t>
+          <t>Lotus pedunculatus</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>Luzcam</t>
+          <t>Lotuli</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>Luzula campestris</t>
+          <t>Lotus uliginosus</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>Luzmul</t>
+          <t>Luzcam</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>Luzula multiflora</t>
+          <t>Luzula campestris</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>Lycflo</t>
+          <t>Luzmul</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>Lycnis flocuculi</t>
+          <t>Luzula multiflora</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>Lysnum</t>
+          <t>Lycflo</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>Lysimachia numularia</t>
+          <t>Lycnis flocuculi</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>Lysvul</t>
+          <t>Lysnum</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>Lysimachia vulgaris</t>
+          <t>Lysimachia numularia</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>Matcha</t>
+          <t>Lysvul</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>Matricaria chamomilla</t>
+          <t>Lysimachia vulgaris</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>Mousse</t>
+          <t>Matcha</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>Mousses</t>
+          <t>Matricaria chamomilla</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>Myodis</t>
+          <t>Mousse</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>Myosotis discolor</t>
+          <t>Mousses</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>Myohis</t>
+          <t>Myodis</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>Myosotis hirsuta</t>
+          <t>Myosotis discolor</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>Myomin</t>
+          <t>Myohis</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>Myosotis minima</t>
+          <t>Myosotis hirsuta</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>Myopal</t>
+          <t>Myomin</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>Myosotis palustris</t>
+          <t>Myosotis minima</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>Myoram</t>
+          <t>Myopal</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>Myosotis ramosissima</t>
+          <t>Myosotis palustris</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>Orcmac</t>
+          <t>Myoram</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>Orchis maculata</t>
+          <t>Myosotis ramosissima</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>Orcmor</t>
+          <t>Orcmac</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>Orchis morio</t>
+          <t>Orchis maculata</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>Phlpra</t>
+          <t>Orcmor</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>Phleum pratense</t>
+          <t>Orchis morio</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>Phraus</t>
+          <t>Phlpra</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>Phragmites australis</t>
+          <t>Phleum pratense</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>Plalan</t>
+          <t>Phraus</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>Plantago lanceolata</t>
+          <t>Phragmites australis</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>Plamaj</t>
+          <t>Plalan</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>Plantago major</t>
+          <t>Plantago lanceolata</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>Poaann</t>
+          <t>Plamaj</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>Poa annua</t>
+          <t>Plantago major</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>Poapra</t>
+          <t>Poaann</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>Poa pratensis</t>
+          <t>Poa annua</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>Poatri</t>
+          <t>Poapra</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>Poa trivialis</t>
+          <t>Poa pratensis</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>Polagu</t>
+          <t>Poatri</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>Poa trivialis</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>Polavi</t>
-        </is>
-      </c>
-      <c r="B121" t="inlineStr">
-        <is>
-          <t>Polygonum aviculare</t>
+          <t>Polagu</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>Potrep</t>
+          <t>Polavi</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>Potentilla reptens</t>
+          <t>Polygonum aviculare</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>Potans</t>
+          <t>Potrep</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>Potentilla repens</t>
+          <t>Potentilla reptens</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>Pouss</t>
+          <t>Potans</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>Potentilla repens</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>Pruspi</t>
-        </is>
-      </c>
-      <c r="B125" t="inlineStr">
-        <is>
-          <t>Prunus spinosa</t>
+          <t>Pouss</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>Ranacr</t>
+          <t>Pruspi</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>Ranunculus acris</t>
+          <t>Prunus spinosa</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>Ranbul</t>
+          <t>Ranacr</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>Ranunculus bulbosus</t>
+          <t>Ranunculus acris</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>Ranfla</t>
+          <t>Ranbul</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>Ranunculus flammula</t>
+          <t>Ranunculus bulbosus</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>Ranrep</t>
+          <t>Ranfla</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>Ranunculus repens</t>
+          <t>Ranunculus flammula</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>Rhimin</t>
+          <t>Ranrep</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>Rhinanthus minor</t>
+          <t>Ranunculus repens</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>Rossp</t>
+          <t>Rhimin</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>Rosa sp.</t>
+          <t>Rhinanthus minor</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>Rubsp</t>
+          <t>Rossp</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>Rubus sp.</t>
+          <t>Rosa sp.</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>Rumace</t>
+          <t>Rubsp</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>Rumex acetosa</t>
+          <t>Rubus sp.</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>Rumacu</t>
+          <t>Rumace</t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>Rumex acutus</t>
+          <t>Rumex acetosa</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>Rumcon</t>
+          <t>Rumacu</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>Rumex conglomeratus</t>
+          <t>Rumex acutus</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>Rumcri</t>
+          <t>Rumcon</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>Rumex crispus</t>
+          <t>Rumex conglomeratus</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>Rumlon</t>
+          <t>Rumcri</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>Rumex longifolius</t>
+          <t>Rumex crispus</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>Rumobt</t>
+          <t>Rumlon</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>Rumex obtusifolius</t>
+          <t>Rumex longifolius</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>Salsp</t>
+          <t>Rumobt</t>
         </is>
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>Salix sp.</t>
+          <t>Rumex obtusifolius</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>Senjac</t>
+          <t>Salsp</t>
         </is>
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>Senecio jacobea</t>
+          <t>Salix sp.</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>Sensp</t>
+          <t>Senjac</t>
         </is>
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>Senecio sp.</t>
+          <t>Senecio jacobea</t>
         </is>
       </c>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>Stegra</t>
+          <t>Sensp</t>
         </is>
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>Stellaria graminea</t>
+          <t>Senecio sp.</t>
         </is>
       </c>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>Stehos</t>
+          <t>Stegra</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>Stelaria holostea</t>
+          <t>Stellaria graminea</t>
         </is>
       </c>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>Stemed</t>
+          <t>Stehos</t>
         </is>
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>Stelaria media</t>
+          <t>Stelaria holostea</t>
         </is>
       </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>Silflo</t>
+          <t>Stemed</t>
         </is>
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>Silene flos-cuculi</t>
+          <t>Stelaria media</t>
         </is>
       </c>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>Taroff</t>
+          <t>Silflo</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>Taraxacum officinalis</t>
+          <t>Silene flos-cuculi</t>
         </is>
       </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>Tarsp</t>
+          <t>Taroff</t>
         </is>
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>Taraxacum sp.</t>
+          <t>Taraxacum officinalis</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>Trapra</t>
+          <t>Tarsp</t>
         </is>
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>Tragopogon pratense</t>
+          <t>Taraxacum sp.</t>
         </is>
       </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>Tridub</t>
+          <t>Trapra</t>
         </is>
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>Trifolium dubium (=Trifolium campestre)</t>
+          <t>Tragopogon pratense</t>
         </is>
       </c>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>Trifla</t>
+          <t>Tridub</t>
         </is>
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>Trisetum flavescens</t>
+          <t>Trifolium dubium (=Trifolium campestre)</t>
         </is>
       </c>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>Tripra</t>
+          <t>Trifla</t>
         </is>
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>Trifolium pratense</t>
+          <t>Trisetum flavescens</t>
         </is>
       </c>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>Trirep</t>
+          <t>Tripra</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>Trifolium repens</t>
+          <t>Trifolium pratense</t>
         </is>
       </c>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>Veralc</t>
+          <t>Trirep</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>Trifolium repens</t>
         </is>
       </c>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>Veraci</t>
-        </is>
-      </c>
-      <c r="B154" t="inlineStr">
-        <is>
-          <t>Veronica acinifolia</t>
+          <t>Veralc</t>
         </is>
       </c>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>Verarv</t>
+          <t>Veraci</t>
         </is>
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>Veronica arvense</t>
+          <t>Veronica acinifolia</t>
         </is>
       </c>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>vercha</t>
+          <t>Veragr</t>
         </is>
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>Veronica chamaedrys</t>
+          <t>Veronica agrestis</t>
         </is>
       </c>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>Verbec</t>
+          <t>Verarv</t>
         </is>
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>Veronica beccabunga</t>
+          <t>Veronica arvense</t>
         </is>
       </c>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>Veroff</t>
+          <t>vercha</t>
         </is>
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>Veronica officinalis</t>
+          <t>Veronica chamaedrys</t>
         </is>
       </c>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>Verper</t>
+          <t>Verbec</t>
         </is>
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>Veronica persica</t>
+          <t>Veronica beccabunga</t>
         </is>
       </c>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>verspi</t>
+          <t>Veroff</t>
         </is>
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>Veronica spicata</t>
+          <t>Veronica officinalis</t>
         </is>
       </c>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>Vicbis</t>
+          <t>Verper</t>
         </is>
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>Vicia bisperma</t>
+          <t>Veronica persica</t>
         </is>
       </c>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>Vichir</t>
+          <t>verspi</t>
         </is>
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>Vicia hirsuta</t>
+          <t>Veronica spicata</t>
         </is>
       </c>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>Viclat</t>
+          <t>Vicbis</t>
         </is>
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>Vicia lathiroides</t>
+          <t>Vicia bisperma</t>
         </is>
       </c>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>Vicsat</t>
+          <t>Vichir</t>
         </is>
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>Vicia sativa</t>
+          <t>Vicia hirsuta</t>
         </is>
       </c>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>Vicsep</t>
+          <t>Viclat</t>
         </is>
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>Vicia sepium</t>
+          <t>Vicia lathiroides</t>
         </is>
       </c>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>Victet</t>
+          <t>Vicsat</t>
         </is>
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>Vicia tetrasperma</t>
+          <t>Vicia sativa</t>
         </is>
       </c>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
+          <t>Vicsep</t>
+        </is>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>Vicia sepium</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>Victet</t>
+        </is>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>Vicia tetrasperma</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
           <t>Vulmyu</t>
         </is>
       </c>
-      <c r="B167" t="inlineStr">
+      <c r="B169" t="inlineStr">
         <is>
           <t>Vulpia myuros</t>
         </is>

</xml_diff>